<commit_message>
Add variables and locations to data dictionary. some variables might be doubled or unnecessary.
</commit_message>
<xml_diff>
--- a/docs/goat_data_dictionary.xlsx
+++ b/docs/goat_data_dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/camilachicatto/2026_startup_goats/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38B75A52-CC69-A743-8EC0-94C5412F20D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB586EF9-EDC7-2A44-8DCD-58BAEE63D859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="680" windowWidth="28040" windowHeight="16920" xr2:uid="{0DF32BC2-826F-6B48-94CE-D6017A50CA52}"/>
+    <workbookView xWindow="11300" yWindow="660" windowWidth="18620" windowHeight="18680" xr2:uid="{0DF32BC2-826F-6B48-94CE-D6017A50CA52}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,143 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="44">
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>width_between_legs</t>
+  </si>
+  <si>
+    <t>hock_height</t>
+  </si>
+  <si>
+    <t>leg_height</t>
+  </si>
+  <si>
+    <t>leg_curve.R</t>
+  </si>
+  <si>
+    <t>udder.curve.R</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>l</t>
+  </si>
+  <si>
+    <t>n_points</t>
+  </si>
+  <si>
+    <t>a_param</t>
+  </si>
+  <si>
+    <t>d_param</t>
+  </si>
+  <si>
+    <t>s_param</t>
+  </si>
+  <si>
+    <t>l_param</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>o</t>
+  </si>
+  <si>
+    <t>u</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>teat_length_score</t>
+  </si>
+  <si>
+    <t>teats_curve.R</t>
+  </si>
+  <si>
+    <t>pelvic.curve.R</t>
+  </si>
+  <si>
+    <t>medial_curve.R</t>
+  </si>
+  <si>
+    <t>ui.teats.R</t>
+  </si>
+  <si>
+    <t>app.R</t>
+  </si>
+  <si>
+    <t>top_y</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>med_o</t>
+  </si>
+  <si>
+    <t>med_p</t>
+  </si>
+  <si>
+    <t>med_q</t>
+  </si>
+  <si>
+    <t>arch_a</t>
+  </si>
+  <si>
+    <t>arch_d</t>
+  </si>
+  <si>
+    <t>arch_s</t>
+  </si>
+  <si>
+    <t>o_param</t>
+  </si>
+  <si>
+    <t>p_param</t>
+  </si>
+  <si>
+    <t>q_param</t>
+  </si>
+  <si>
+    <t>r_param</t>
+  </si>
+  <si>
+    <t>j_param</t>
+  </si>
+  <si>
+    <t>u_param</t>
+  </si>
+  <si>
+    <t>h_param</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -405,9 +542,482 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99C34CDA-7263-D04D-BE92-B36483DF3D5D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="2" width="25.33203125" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" customWidth="1"/>
+    <col min="4" max="4" width="96" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>38</v>
+      </c>
+      <c r="B38" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>16</v>
+      </c>
+      <c r="B40" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>18</v>
+      </c>
+      <c r="B43" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>19</v>
+      </c>
+      <c r="B44" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>16</v>
+      </c>
+      <c r="B48" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>14</v>
+      </c>
+      <c r="B50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>13</v>
+      </c>
+      <c r="B51" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>15</v>
+      </c>
+      <c r="B52" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>37</v>
+      </c>
+      <c r="B53" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>38</v>
+      </c>
+      <c r="B54" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>39</v>
+      </c>
+      <c r="B55" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>41</v>
+      </c>
+      <c r="B56" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>42</v>
+      </c>
+      <c r="B57" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>43</v>
+      </c>
+      <c r="B58" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update data dictionary, filled more definitions and alphabetized
</commit_message>
<xml_diff>
--- a/docs/goat_data_dictionary.xlsx
+++ b/docs/goat_data_dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/camilachicatto/2026_startup_goats/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A00868-7A79-774F-95A8-361C11A10CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746E5C7B-2E65-4B4F-AB4C-D5C8CEB65974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8500" yWindow="660" windowWidth="21420" windowHeight="18680" xr2:uid="{0DF32BC2-826F-6B48-94CE-D6017A50CA52}"/>
+    <workbookView xWindow="500" yWindow="840" windowWidth="29260" windowHeight="16620" xr2:uid="{0DF32BC2-826F-6B48-94CE-D6017A50CA52}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="49">
   <si>
     <t>Definition</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Location</t>
   </si>
   <si>
-    <t>width_between_legs</t>
-  </si>
-  <si>
     <t>hock_height</t>
   </si>
   <si>
@@ -62,27 +59,9 @@
     <t>leg_curve.R</t>
   </si>
   <si>
-    <t>l</t>
-  </si>
-  <si>
     <t>n_points</t>
   </si>
   <si>
-    <t>j</t>
-  </si>
-  <si>
-    <t>q</t>
-  </si>
-  <si>
-    <t>o</t>
-  </si>
-  <si>
-    <t>u</t>
-  </si>
-  <si>
-    <t>h</t>
-  </si>
-  <si>
     <t>teat_length_score</t>
   </si>
   <si>
@@ -92,9 +71,6 @@
     <t>medial_curve.R</t>
   </si>
   <si>
-    <t>app.R</t>
-  </si>
-  <si>
     <t>top_y</t>
   </si>
   <si>
@@ -143,9 +119,6 @@
     <t>bot_y</t>
   </si>
   <si>
-    <t xml:space="preserve">Controls the amount of space between the legs. Defined as the space between the inner boundary line of the two legs. </t>
-  </si>
-  <si>
     <t>Controls the distance between the ground and the hock, or the rear knee joint.</t>
   </si>
   <si>
@@ -158,12 +131,6 @@
     <t>width scaling of the teat</t>
   </si>
   <si>
-    <t>horizontal boundary for the plot x-range</t>
-  </si>
-  <si>
-    <t>horizontal distance between the legs, constrained to 0–20 inches</t>
-  </si>
-  <si>
     <t>Closed polygon for the region above the pelvic arch, capped at top_y</t>
   </si>
   <si>
@@ -173,12 +140,6 @@
     <t>depth/curvature of the medial suspensory ligament</t>
   </si>
   <si>
-    <t>horizontal distance between the legs</t>
-  </si>
-  <si>
-    <t>height of the rear knee joint above the ground baseline</t>
-  </si>
-  <si>
     <t xml:space="preserve">Controls the curvature and steepness of the udder arch. Relates to "a" variable in Desmos. </t>
   </si>
   <si>
@@ -188,12 +149,6 @@
     <t>Controls the distance from the midline of the udder (think the highest point of the medial) to each teat. Correlates to the "j" variable in Desmos. When this variable is zero, the teats are so close together only half of a teat shows up right on the midline of the udder, creating the illusion of a singular teat right on the midline of the udder in a cyclops fashion.</t>
   </si>
   <si>
-    <t>leg_curve.R, udder_curve.R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controls the amount of space between the legs. Defined as the space between the inner boundary line of the two legs. In the udder_arch.R script, it affects the horizontal span of the udder arch. </t>
-  </si>
-  <si>
     <t>medial_curve.R, pelvic_curve.R, teats_curve.R, udder_curve.R</t>
   </si>
   <si>
@@ -203,25 +158,53 @@
     <t>Sets the distance between parabola roots (where the arms of the parabola, or teat, crosses the x axis); controls teat width. Correlates to "h" variable in Desmos.</t>
   </si>
   <si>
-    <t>medial_curve.R, teats_curve.R</t>
-  </si>
-  <si>
     <t>where the udder floor sits (shared with medial). height of the udder floor above the ground baseline</t>
   </si>
   <si>
     <t>Determines the length of the teat; the distance between the tip of the teat and the udder floor.</t>
+  </si>
+  <si>
+    <t>app. R, teats_curve.R</t>
+  </si>
+  <si>
+    <t>app. R, medial_curve.R, teats_curve.R</t>
+  </si>
+  <si>
+    <t>app. R, udder_curve.R</t>
+  </si>
+  <si>
+    <t>app.R, udder_curve.R</t>
+  </si>
+  <si>
+    <t>app.R, leg_curve.R, medial_curve.R</t>
+  </si>
+  <si>
+    <t>app. R,medial_curve.R, teats_curve.R</t>
+  </si>
+  <si>
+    <t>app.R, leg_curve.R, medial_curve.R, pelvic_curve.R, teats_curve.R, udder_curve.R</t>
+  </si>
+  <si>
+    <t>Controls the amount of space between the legs. Defined as the space between the inner boundary line of the two legs. In the udder_arch.R script, it affects the horizontal span of the udder arch. Values limited to 0 to 20 inches. Teats: horizontal boundary for the plot x-range</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -245,8 +228,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99C34CDA-7263-D04D-BE92-B36483DF3D5D}">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="25.33203125" customWidth="1"/>
@@ -589,23 +573,23 @@
     <col min="4" max="4" width="23.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="C2" t="s">
         <v>34</v>
@@ -613,59 +597,56 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>43</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -673,10 +654,10 @@
         <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -684,40 +665,40 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
         <v>48</v>
@@ -725,222 +706,109 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>15</v>
+        <v>41</v>
+      </c>
+      <c r="C19" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>15</v>
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>4</v>
-      </c>
-      <c r="B27" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>22</v>
-      </c>
-      <c r="B28" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>24</v>
-      </c>
-      <c r="B30" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>9</v>
-      </c>
-      <c r="B31" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>10</v>
-      </c>
-      <c r="B32" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
         <v>11</v>
       </c>
-      <c r="B33" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>12</v>
-      </c>
-      <c r="B34" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>13</v>
-      </c>
-      <c r="B35" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36" t="s">
-        <v>17</v>
-      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C23">
+    <sortCondition ref="A2:A23"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update dictionary, things in red still need revision
</commit_message>
<xml_diff>
--- a/docs/goat_data_dictionary.xlsx
+++ b/docs/goat_data_dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/camilachicatto/2026_startup_goats/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746E5C7B-2E65-4B4F-AB4C-D5C8CEB65974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BBF273-DF53-0541-B771-92088DB620F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="500" yWindow="840" windowWidth="29260" windowHeight="16620" xr2:uid="{0DF32BC2-826F-6B48-94CE-D6017A50CA52}"/>
+    <workbookView xWindow="15160" yWindow="660" windowWidth="14760" windowHeight="18680" xr2:uid="{0DF32BC2-826F-6B48-94CE-D6017A50CA52}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="46">
   <si>
     <t>Definition</t>
   </si>
@@ -68,21 +68,12 @@
     <t>teats_curve.R</t>
   </si>
   <si>
-    <t>medial_curve.R</t>
-  </si>
-  <si>
     <t>top_y</t>
   </si>
   <si>
-    <t>udder_curve.R</t>
-  </si>
-  <si>
     <t>pelvic_curve.R</t>
   </si>
   <si>
-    <t>x</t>
-  </si>
-  <si>
     <t>arch_roundness</t>
   </si>
   <si>
@@ -170,12 +161,6 @@
     <t>app. R, medial_curve.R, teats_curve.R</t>
   </si>
   <si>
-    <t>app. R, udder_curve.R</t>
-  </si>
-  <si>
-    <t>app.R, udder_curve.R</t>
-  </si>
-  <si>
     <t>app.R, leg_curve.R, medial_curve.R</t>
   </si>
   <si>
@@ -186,13 +171,19 @@
   </si>
   <si>
     <t>Controls the amount of space between the legs. Defined as the space between the inner boundary line of the two legs. In the udder_arch.R script, it affects the horizontal span of the udder arch. Values limited to 0 to 20 inches. Teats: horizontal boundary for the plot x-range</t>
+  </si>
+  <si>
+    <t>app.R, medial_curve.R, udder_curve.R</t>
+  </si>
+  <si>
+    <t>app. R, medial_curve.R, udder_curve.R</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -205,6 +196,13 @@
       <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -228,9 +226,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -565,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99C34CDA-7263-D04D-BE92-B36483DF3D5D}">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="25.33203125" customWidth="1"/>
@@ -586,228 +585,199 @@
     </row>
     <row r="2" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
         <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" t="s">
-        <v>33</v>
+      <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
+      <c r="A5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
         <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" t="s">
-        <v>37</v>
-      </c>
+      <c r="A14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" t="s">
-        <v>8</v>
-      </c>
+      <c r="A17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" t="s">
-        <v>35</v>
+      <c r="A18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" t="s">
-        <v>41</v>
-      </c>
-      <c r="C19" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>10</v>
-      </c>
-      <c r="B20" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="A19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23" t="s">
-        <v>11</v>
+      <c r="C19" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C23">
-    <sortCondition ref="A2:A23"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C20">
+    <sortCondition ref="A2:A20"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>